<commit_message>
adjusted decodeKey logic (last [bracket] is used for groups)
</commit_message>
<xml_diff>
--- a/templates/GLL_template.xlsx
+++ b/templates/GLL_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="1" state="visible" r:id="rId3"/>
@@ -45,7 +45,7 @@
     <t xml:space="preserve">User Data [group]</t>
   </si>
   <si>
-    <t xml:space="preserve">Add any user-defined property as a new column. For logical grouping, put your category in [brackets] (e.g. node property “property A” that belongs to the group “group A”).</t>
+    <t xml:space="preserve">Add custom properties in new columns. Use [brackets] for grouping (e.g., "Temperature [Celsius] [Physics]"). The last [bracket] becomes the group name.</t>
   </si>
   <si>
     <t xml:space="preserve">Data Types Explained</t>
@@ -204,7 +204,7 @@
     <t xml:space="preserve">property A [group A]</t>
   </si>
   <si>
-    <t xml:space="preserve">User-defined node properties</t>
+    <t xml:space="preserve">User-defined custom node properties</t>
   </si>
   <si>
     <t xml:space="preserve">Edge Properties Explained</t>
@@ -351,13 +351,13 @@
     <t xml:space="preserve">The stroke width of the halo</t>
   </si>
   <si>
-    <t xml:space="preserve">User-defined edge properties</t>
+    <t xml:space="preserve">User-defined custom edge properties</t>
   </si>
   <si>
     <t xml:space="preserve">Feature X [group A]</t>
   </si>
   <si>
-    <t xml:space="preserve">Feature Y [group A]</t>
+    <t xml:space="preserve">Feature Y [nm] [group A]</t>
   </si>
   <si>
     <t xml:space="preserve">Feature Z [group B]</t>
@@ -910,7 +910,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="136.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="122.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="15.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="98.86"/>
   </cols>
@@ -1635,7 +1635,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="19.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="19.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="19.73"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="25" width="11.53"/>
   </cols>

</xml_diff>

<commit_message>
KG-230: Added Excel export in Data Editor
</commit_message>
<xml_diff>
--- a/templates/GLL_template.xlsx
+++ b/templates/GLL_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="141">
   <si>
     <t xml:space="preserve">Color Codes Explained</t>
   </si>
@@ -108,6 +108,12 @@
     <t xml:space="preserve">text (unique)</t>
   </si>
   <si>
+    <t xml:space="preserve">Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Label of the node; if no Label is given, the ID is displayed per default</t>
+  </si>
+  <si>
     <t xml:space="preserve">Description of the node, displayed in the tooltip text</t>
   </si>
   <si>
@@ -153,12 +159,6 @@
     <t xml:space="preserve">The stroke color of the node in RGBA format</t>
   </si>
   <si>
-    <t xml:space="preserve">Label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Label of the node; if no Label is given, the ID is displayed per default</t>
-  </si>
-  <si>
     <t xml:space="preserve">Label Font Size</t>
   </si>
   <si>
@@ -222,6 +222,12 @@
     <t xml:space="preserve">The ID of the target node</t>
   </si>
   <si>
+    <t xml:space="preserve">Label of the edge; if no Label is given, the edge is only visible as line without any text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description of the edge, displayed in the tooltip text</t>
+  </si>
+  <si>
     <t xml:space="preserve">The edge type</t>
   </si>
   <si>
@@ -250,9 +256,6 @@
   </si>
   <si>
     <t xml:space="preserve">#403C5390</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Label of the edge; if no Label is given, the edge is only visible as line without any text</t>
   </si>
   <si>
     <t xml:space="preserve">The font size of the edges label</t>
@@ -452,7 +455,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -504,6 +507,11 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <u val="single"/>
       <sz val="10"/>
       <name val="Arial"/>
@@ -543,7 +551,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -555,13 +563,6 @@
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin"/>
       <diagonal/>
     </border>
@@ -598,7 +599,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -627,16 +628,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -651,10 +648,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -663,11 +656,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -679,19 +672,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -906,7 +899,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.06"/>
@@ -968,16 +961,16 @@
         <v>7</v>
       </c>
       <c r="C4" s="8"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -987,75 +980,75 @@
       <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="11"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="14"/>
+      <c r="C7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="14"/>
+      <c r="C8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="14"/>
+      <c r="C9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="14"/>
+      <c r="C10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="14"/>
+      <c r="C11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="14"/>
+      <c r="C12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1075,10 +1068,10 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>26</v>
@@ -1089,30 +1082,30 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>32</v>
+        <v>26</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="D18" s="16" t="s">
         <v>34</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1122,25 +1115,25 @@
       <c r="B19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>38</v>
+      <c r="C19" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="D20" s="17" t="s">
         <v>40</v>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1150,11 +1143,11 @@
       <c r="B21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D21" s="19" t="s">
-        <v>38</v>
+      <c r="C21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1167,8 +1160,8 @@
       <c r="C22" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>9</v>
+      <c r="D22" s="17" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1195,7 +1188,7 @@
       <c r="C24" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="16" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1209,8 +1202,8 @@
       <c r="C25" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="19" t="s">
-        <v>38</v>
+      <c r="D25" s="17" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1223,8 +1216,8 @@
       <c r="C26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="19" t="s">
-        <v>38</v>
+      <c r="D26" s="17" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1262,7 +1255,7 @@
       <c r="B29" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="8" t="s">
         <v>26</v>
       </c>
       <c r="D29" s="7" t="s">
@@ -1270,20 +1263,20 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="19"/>
-      <c r="C30" s="21"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="18"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D31" s="16" t="s">
+      <c r="D31" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1291,13 +1284,13 @@
       <c r="A32" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="19" t="s">
+      <c r="D32" s="17" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1305,310 +1298,324 @@
       <c r="A33" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="C33" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D33" s="19" t="s">
+      <c r="D33" s="17" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B34" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="C34" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D34" s="18" t="s">
-        <v>68</v>
+      <c r="C34" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34" s="17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="C35" s="21" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D35" s="19" t="s">
-        <v>11</v>
+        <v>67</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B36" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="C36" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="19" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B37" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="D37" s="19" t="s">
-        <v>38</v>
+        <v>71</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B38" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="D38" s="19" t="s">
-        <v>9</v>
+        <v>73</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B39" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="C39" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>11</v>
+      <c r="D39" s="17" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B40" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C40" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="C40" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="D40" s="18" t="s">
-        <v>81</v>
+      <c r="D40" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B41" s="19" t="s">
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C41" s="22" t="n">
+      <c r="B42" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="C42" s="20" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D41" s="19" t="s">
+      <c r="D42" s="17" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B42" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="C42" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="19" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="B43" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="C43" s="21" t="n">
+      <c r="C43" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D43" s="19" t="s">
+      <c r="D43" s="17" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B44" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C44" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="D44" s="19" t="s">
-        <v>38</v>
+      <c r="C44" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="17" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B45" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B45" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="C45" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D45" s="19" t="s">
-        <v>38</v>
+      <c r="C45" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45" s="17" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B46" s="19" t="s">
+      <c r="D46" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C46" s="22" t="n">
+      <c r="B47" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="C47" s="20" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D46" s="19" t="s">
+      <c r="D47" s="17" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B47" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="C47" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D47" s="19" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="B48" s="19" t="s">
-        <v>96</v>
-      </c>
-      <c r="C48" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="D48" s="18" t="s">
-        <v>98</v>
+      <c r="C48" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" s="17" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="C49" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="D49" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="B49" s="19" t="s">
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C49" s="22" t="n">
+      <c r="B50" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="C50" s="20" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D49" s="19" t="s">
+      <c r="D50" s="17" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B50" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="C50" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D50" s="23" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B51" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="B51" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C51" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="D51" s="18" t="s">
-        <v>98</v>
+      <c r="C51" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D51" s="21" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B52" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="B52" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="C52" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D52" s="19" t="s">
-        <v>38</v>
+      <c r="C52" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="D52" s="16" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B53" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="B53" s="24" t="s">
+      <c r="C53" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="D53" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C53" s="21" t="n">
+      <c r="B54" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="C54" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D53" s="19" t="s">
+      <c r="D54" s="17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="6" t="s">
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B54" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="C54" s="21" t="s">
+      <c r="B55" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C55" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D54" s="19" t="s">
+      <c r="D55" s="17" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1628,7 +1635,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N1006"/>
+  <dimension ref="A1:P1006"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.2"/>
@@ -1638,7 +1645,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="19.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="19.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="25" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="23" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1646,174 +1653,174 @@
         <v>24</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
-        <v>113</v>
-      </c>
-      <c r="B2" s="27" t="s">
+      <c r="A2" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="B2" s="25" t="s">
         <v>115</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="C2" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="E2" s="28" t="n">
+      <c r="D2" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="E2" s="26" t="n">
         <v>60</v>
       </c>
-      <c r="F2" s="28" t="s">
-        <v>117</v>
-      </c>
-      <c r="G2" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="H2" s="29" t="n">
+      <c r="F2" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="H2" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="J2" s="29" t="n">
+      <c r="I2" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="J2" s="27" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="25"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I3" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>121</v>
-      </c>
-      <c r="D3" s="27"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="29" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I3" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="J3" s="29" t="n">
+      <c r="J3" s="27" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4" s="27" t="s">
+      <c r="A4" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="B4" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="29" t="n">
+      <c r="C4" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="27" t="n">
         <v>1.1</v>
       </c>
-      <c r="I4" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="J4" s="29" t="n">
+      <c r="I4" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="J4" s="27" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="27" t="s">
+      <c r="A5" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="B5" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="29" t="n">
+      <c r="C5" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5" s="25"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="27" t="n">
         <v>1.3</v>
       </c>
-      <c r="I5" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="J5" s="29" t="n">
+      <c r="I5" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="J5" s="27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" s="25"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="27" t="s">
         <v>129</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="J6" s="29" t="n">
+      <c r="J6" s="27" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="B7" s="27" t="s">
+      <c r="A7" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="29" t="n">
+      <c r="B7" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="27" t="n">
         <v>-1</v>
       </c>
-      <c r="I7" s="29"/>
-      <c r="J7" s="29"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2739,20 +2746,160 @@
     <row r="929" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="930" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="931" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="932" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="933" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="934" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="935" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="936" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="937" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="938" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="939" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="940" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="941" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="942" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="943" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="944" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="945" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="932" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B932" s="1"/>
+      <c r="D932" s="1"/>
+      <c r="E932" s="1"/>
+      <c r="K932" s="1"/>
+      <c r="L932" s="1"/>
+      <c r="M932" s="1"/>
+      <c r="N932" s="1"/>
+      <c r="O932" s="1"/>
+      <c r="P932" s="1"/>
+    </row>
+    <row r="933" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B933" s="1"/>
+      <c r="D933" s="1"/>
+      <c r="E933" s="1"/>
+      <c r="K933" s="1"/>
+      <c r="L933" s="1"/>
+      <c r="M933" s="1"/>
+      <c r="N933" s="1"/>
+      <c r="O933" s="1"/>
+      <c r="P933" s="1"/>
+    </row>
+    <row r="934" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B934" s="1"/>
+      <c r="D934" s="1"/>
+      <c r="E934" s="1"/>
+      <c r="K934" s="1"/>
+      <c r="L934" s="1"/>
+      <c r="M934" s="1"/>
+      <c r="N934" s="1"/>
+      <c r="O934" s="1"/>
+      <c r="P934" s="1"/>
+    </row>
+    <row r="935" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B935" s="1"/>
+      <c r="D935" s="1"/>
+      <c r="E935" s="1"/>
+      <c r="K935" s="1"/>
+      <c r="L935" s="1"/>
+      <c r="M935" s="1"/>
+      <c r="N935" s="1"/>
+      <c r="O935" s="1"/>
+      <c r="P935" s="1"/>
+    </row>
+    <row r="936" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B936" s="1"/>
+      <c r="D936" s="1"/>
+      <c r="E936" s="1"/>
+      <c r="K936" s="1"/>
+      <c r="L936" s="1"/>
+      <c r="M936" s="1"/>
+      <c r="N936" s="1"/>
+      <c r="O936" s="1"/>
+      <c r="P936" s="1"/>
+    </row>
+    <row r="937" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B937" s="1"/>
+      <c r="D937" s="1"/>
+      <c r="E937" s="1"/>
+      <c r="K937" s="1"/>
+      <c r="L937" s="1"/>
+      <c r="M937" s="1"/>
+      <c r="N937" s="1"/>
+      <c r="O937" s="1"/>
+      <c r="P937" s="1"/>
+    </row>
+    <row r="938" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B938" s="1"/>
+      <c r="D938" s="1"/>
+      <c r="E938" s="1"/>
+      <c r="K938" s="1"/>
+      <c r="L938" s="1"/>
+      <c r="M938" s="1"/>
+      <c r="N938" s="1"/>
+      <c r="O938" s="1"/>
+      <c r="P938" s="1"/>
+    </row>
+    <row r="939" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B939" s="1"/>
+      <c r="D939" s="1"/>
+      <c r="E939" s="1"/>
+      <c r="K939" s="1"/>
+      <c r="L939" s="1"/>
+      <c r="M939" s="1"/>
+      <c r="N939" s="1"/>
+      <c r="O939" s="1"/>
+      <c r="P939" s="1"/>
+    </row>
+    <row r="940" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B940" s="1"/>
+      <c r="D940" s="1"/>
+      <c r="E940" s="1"/>
+      <c r="K940" s="1"/>
+      <c r="L940" s="1"/>
+      <c r="M940" s="1"/>
+      <c r="N940" s="1"/>
+      <c r="O940" s="1"/>
+      <c r="P940" s="1"/>
+    </row>
+    <row r="941" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B941" s="1"/>
+      <c r="D941" s="1"/>
+      <c r="E941" s="1"/>
+      <c r="K941" s="1"/>
+      <c r="L941" s="1"/>
+      <c r="M941" s="1"/>
+      <c r="N941" s="1"/>
+      <c r="O941" s="1"/>
+      <c r="P941" s="1"/>
+    </row>
+    <row r="942" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B942" s="1"/>
+      <c r="D942" s="1"/>
+      <c r="E942" s="1"/>
+      <c r="K942" s="1"/>
+      <c r="L942" s="1"/>
+      <c r="M942" s="1"/>
+      <c r="N942" s="1"/>
+      <c r="O942" s="1"/>
+      <c r="P942" s="1"/>
+    </row>
+    <row r="943" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B943" s="1"/>
+      <c r="D943" s="1"/>
+      <c r="E943" s="1"/>
+      <c r="K943" s="1"/>
+      <c r="L943" s="1"/>
+      <c r="M943" s="1"/>
+      <c r="N943" s="1"/>
+      <c r="O943" s="1"/>
+      <c r="P943" s="1"/>
+    </row>
+    <row r="944" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B944" s="1"/>
+      <c r="D944" s="1"/>
+      <c r="E944" s="1"/>
+      <c r="K944" s="1"/>
+      <c r="L944" s="1"/>
+      <c r="M944" s="1"/>
+      <c r="N944" s="1"/>
+      <c r="O944" s="1"/>
+      <c r="P944" s="1"/>
+    </row>
+    <row r="945" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B945" s="1"/>
+      <c r="D945" s="1"/>
+      <c r="E945" s="1"/>
+      <c r="K945" s="1"/>
+      <c r="L945" s="1"/>
+      <c r="M945" s="1"/>
+      <c r="N945" s="1"/>
+      <c r="O945" s="1"/>
+      <c r="P945" s="1"/>
+    </row>
     <row r="946" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B946" s="1"/>
       <c r="D946" s="1"/>
@@ -3317,119 +3464,119 @@
         <v>64</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
-        <v>113</v>
-      </c>
-      <c r="B2" s="26" t="s">
+      <c r="A2" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" s="25" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="C2" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="D2" s="27" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="F2" s="29" t="n">
+      <c r="F2" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="29" t="s">
-        <v>136</v>
-      </c>
-      <c r="H2" s="29" t="n">
+      <c r="G2" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="H2" s="27" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>113</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="29" t="n">
+      <c r="A3" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="27" t="n">
         <v>0.5</v>
       </c>
-      <c r="G3" s="29" t="s">
-        <v>137</v>
-      </c>
-      <c r="H3" s="29" t="n">
+      <c r="G3" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="H3" s="27" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>125</v>
-      </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="29" t="n">
+      <c r="A4" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="27" t="n">
         <v>1.1</v>
       </c>
-      <c r="G4" s="29" t="s">
-        <v>138</v>
-      </c>
-      <c r="H4" s="29" t="n">
+      <c r="G4" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="H4" s="27" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="29" t="n">
+      <c r="A5" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="27" t="n">
         <v>1.3</v>
       </c>
-      <c r="G5" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="H5" s="29" t="n">
+      <c r="G5" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="H5" s="27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>